<commit_message>
Update product data files with new entries and sizes in done.txt and input.csv. Enhance error_debug.txt with updated timestamps and processing details. Improve diagnostics in save_diagnostics.log and translation_errors.log for better error tracking and handling. Refactor MagentoFiller to include robust error detection for product save results and recovery mechanisms for failed submissions.
</commit_message>
<xml_diff>
--- a/Casamoda/prijzen.xlsx
+++ b/Casamoda/prijzen.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\info\Downloads\Test prodyct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A34F293-7F00-48AA-A503-294C52DED6F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16D974B1-15BD-4928-8E70-E5E0C51B022B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2280" yWindow="3030" windowWidth="38010" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10230" yWindow="2115" windowWidth="38010" windowHeight="17820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Prijzen" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Prijzen!$A$1:$A$1014</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Prijzen!$A$1:$A$1016</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -346,7 +346,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B1014"/>
+  <dimension ref="A1:B1016"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1531,7 +1531,7 @@
     </row>
     <row r="148" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A148" s="4">
-        <v>33</v>
+        <v>32.799999999999997</v>
       </c>
       <c r="B148" s="7">
         <v>89.99</v>
@@ -1539,17 +1539,17 @@
     </row>
     <row r="149" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A149" s="4">
-        <v>33.9</v>
+        <v>33</v>
       </c>
       <c r="B149" s="7">
         <v>89.99</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A150" s="3">
-        <v>34.65</v>
-      </c>
-      <c r="B150" s="3">
+      <c r="A150" s="4">
+        <v>33.9</v>
+      </c>
+      <c r="B150" s="7">
         <v>89.99</v>
       </c>
     </row>
@@ -1570,114 +1570,114 @@
       </c>
     </row>
     <row r="153" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="2">
+      <c r="A153" s="3">
         <v>34.65</v>
       </c>
-      <c r="B153" s="2">
+      <c r="B153" s="3">
         <v>89.99</v>
       </c>
     </row>
     <row r="154" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154" s="4">
-        <v>36.65</v>
-      </c>
-      <c r="B154" s="7">
-        <v>99.99</v>
+      <c r="A154" s="2">
+        <v>34.65</v>
+      </c>
+      <c r="B154" s="2">
+        <v>89.99</v>
       </c>
     </row>
     <row r="155" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A155" s="4">
-        <v>37</v>
+        <v>35.799999999999997</v>
       </c>
       <c r="B155" s="7">
         <v>99.99</v>
       </c>
     </row>
     <row r="156" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A156" s="2">
+      <c r="A156" s="4">
+        <v>36.65</v>
+      </c>
+      <c r="B156" s="7">
+        <v>99.99</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A157" s="4">
+        <v>37</v>
+      </c>
+      <c r="B157" s="7">
+        <v>99.99</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A158" s="2">
         <v>38.5</v>
       </c>
-      <c r="B156" s="2">
+      <c r="B158" s="2">
         <v>99.99</v>
       </c>
     </row>
-    <row r="157" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157" s="2">
+    <row r="159" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A159" s="2">
         <v>38.5</v>
       </c>
-      <c r="B157" s="2">
+      <c r="B159" s="2">
         <v>99.99</v>
       </c>
     </row>
-    <row r="158" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158" s="4">
+    <row r="160" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A160" s="4">
         <v>40.35</v>
       </c>
-      <c r="B158" s="7">
+      <c r="B160" s="7">
         <v>109.99</v>
       </c>
     </row>
-    <row r="159" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159" s="3">
+    <row r="161" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A161" s="3">
         <v>46.15</v>
       </c>
-      <c r="B159" s="3">
+      <c r="B161" s="3">
         <v>119.99</v>
       </c>
     </row>
-    <row r="160" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A160" s="3">
+    <row r="162" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A162" s="3">
         <v>46.15</v>
       </c>
-      <c r="B160" s="3">
-        <v>119.99</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A161" s="2">
-        <v>46.15</v>
-      </c>
-      <c r="B161" s="2">
-        <v>119.99</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="2">
-        <v>46.15</v>
-      </c>
-      <c r="B162" s="2">
+      <c r="B162" s="3">
         <v>119.99</v>
       </c>
     </row>
     <row r="163" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A163" s="2">
+        <v>46.15</v>
+      </c>
+      <c r="B163" s="2">
+        <v>119.99</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A164" s="2">
+        <v>46.15</v>
+      </c>
+      <c r="B164" s="2">
+        <v>119.99</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A165" s="2">
         <v>57.65</v>
       </c>
-      <c r="B163" s="2">
+      <c r="B165" s="2">
         <v>149.99</v>
       </c>
     </row>
-    <row r="164" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A164" s="3">
+    <row r="166" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A166" s="3">
         <v>57.65</v>
       </c>
-      <c r="B164" s="3">
-        <v>149.99</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="6">
-        <v>57.65</v>
-      </c>
-      <c r="B165" s="6">
-        <v>149.99</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="5">
-        <v>57.65</v>
-      </c>
-      <c r="B166" s="5">
+      <c r="B166" s="3">
         <v>149.99</v>
       </c>
     </row>
@@ -1691,30 +1691,44 @@
     </row>
     <row r="168" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A168" s="5">
-        <v>61.55</v>
+        <v>57.65</v>
       </c>
       <c r="B168" s="5">
-        <v>159.99</v>
+        <v>149.99</v>
       </c>
     </row>
     <row r="169" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A169" s="6">
-        <v>65.400000000000006</v>
+        <v>57.65</v>
       </c>
       <c r="B169" s="6">
-        <v>169.99</v>
+        <v>149.99</v>
       </c>
     </row>
     <row r="170" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A170" s="5">
+        <v>61.55</v>
+      </c>
+      <c r="B170" s="5">
+        <v>159.99</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A171" s="6">
         <v>65.400000000000006</v>
       </c>
-      <c r="B170" s="5">
+      <c r="B171" s="6">
         <v>169.99</v>
       </c>
     </row>
-    <row r="171" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="172" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A172" s="5">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="B172" s="5">
+        <v>169.99</v>
+      </c>
+    </row>
     <row r="173" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="174" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="175" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2557,10 +2571,12 @@
     <row r="1012" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1013" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1014" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1015" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1016" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:A1014" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B1014">
-      <sortCondition ref="A1:A1014"/>
+  <autoFilter ref="A1:A1016" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B1016">
+      <sortCondition ref="A1:A1016"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>

</xml_diff>